<commit_message>
update ash docs and sector parameters
</commit_message>
<xml_diff>
--- a/data/sector_mapping.xlsx
+++ b/data/sector_mapping.xlsx
@@ -56,9 +56,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -492,7 +498,6 @@
           <t>半导体及元件</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>芯片设计、制造、封测</t>
@@ -515,7 +520,6 @@
           <t>计算机应用</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>AI、大模型、智能应用</t>
@@ -538,7 +542,6 @@
           <t>计算机应用</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>云服务、SaaS、数据中心</t>
@@ -561,7 +564,6 @@
           <t>计算机应用</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>软件开发、应用软件</t>
@@ -584,7 +586,6 @@
           <t>传媒</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
           <t>互联网平台、内容</t>
@@ -607,7 +608,6 @@
           <t>计算机应用</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
           <t>IT服务、系统集成</t>
@@ -630,7 +630,6 @@
           <t>电子</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
           <t>电子元器件、面板、PCB</t>
@@ -653,7 +652,6 @@
           <t>电力设备</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
           <t>光伏、风电、储能</t>
@@ -676,7 +674,6 @@
           <t>汽车整车</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
           <t>新能源汽车整车制造</t>
@@ -699,7 +696,6 @@
           <t>电力设备</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
           <t>锂电池制造、材料</t>
@@ -722,7 +718,6 @@
           <t>电力设备</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
           <t>光伏产业链</t>
@@ -745,7 +740,6 @@
           <t>银行</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
           <t>商业银行</t>
@@ -768,7 +762,6 @@
           <t>保险及其他</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
           <t>保险行业</t>
@@ -791,7 +784,6 @@
           <t>证券</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
           <t>证券行业</t>
@@ -814,7 +806,6 @@
           <t>医疗器械</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
           <t>生物技术、创新药</t>
@@ -837,7 +828,6 @@
           <t>医药</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
           <t>制药、医药服务</t>
@@ -860,7 +850,6 @@
           <t>医疗器械</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
           <t>医疗设备、耗材</t>
@@ -883,7 +872,6 @@
           <t>零售</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
           <t>消费品零售</t>
@@ -906,7 +894,6 @@
           <t>食品饮料</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
           <t>食品饮料行业</t>
@@ -929,7 +916,6 @@
           <t>零售</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
           <t>电子商务</t>
@@ -952,7 +938,6 @@
           <t>国防军工</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
           <t>航空航天产业链</t>
@@ -975,7 +960,6 @@
           <t>国防军工</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
           <t>国防军事工业</t>
@@ -998,7 +982,6 @@
           <t>自动化设备</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
           <t>工业机器人、自动化</t>
@@ -1021,7 +1004,6 @@
           <t>油气</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
           <t>石油、天然气勘探开发</t>
@@ -1044,7 +1026,6 @@
           <t>有色金属</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
           <t>有色金属采掘冶炼</t>
@@ -1067,7 +1048,6 @@
           <t>钢铁</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
           <t>钢铁冶炼加工</t>
@@ -1090,7 +1070,6 @@
           <t>煤炭</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
           <t>煤炭开采</t>
@@ -1113,7 +1092,6 @@
           <t>建筑装饰</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
           <t>基础设施建设</t>
@@ -1136,7 +1114,6 @@
           <t>房地产</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
           <t>房地产开发</t>
@@ -1159,7 +1136,6 @@
           <t>物流</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
           <t>物流、快递、航运</t>
@@ -1182,7 +1158,6 @@
           <t>猪肉</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
           <t>US pork futures vs China pork sector</t>
@@ -1205,7 +1180,6 @@
           <t>猪肉</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
           <t>US lean hogs vs China pork</t>
@@ -1385,7 +1359,6 @@
           <t>sz300661</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="n">
         <v>0.2</v>
       </c>
@@ -1406,7 +1379,6 @@
           <t>sz300782</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="n">
         <v>0.2</v>
       </c>
@@ -1427,7 +1399,6 @@
           <t>sh603986</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="n">
         <v>0.2</v>
       </c>
@@ -1448,7 +1419,6 @@
           <t>sz002371</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
         <v>0.2</v>
       </c>
@@ -1469,7 +1439,6 @@
           <t>sz300604</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="n">
         <v>0.2</v>
       </c>
@@ -1490,7 +1459,6 @@
           <t>sz300418</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
       <c r="E7" t="n">
         <v>0.2</v>
       </c>
@@ -1511,7 +1479,6 @@
           <t>sz300624</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
       <c r="E8" t="n">
         <v>0.2</v>
       </c>
@@ -1532,7 +1499,6 @@
           <t>sh603019</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
       <c r="E9" t="n">
         <v>0.2</v>
       </c>
@@ -1553,7 +1519,6 @@
           <t>sz002230</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
       <c r="E10" t="n">
         <v>0.2</v>
       </c>
@@ -1574,7 +1539,6 @@
           <t>sz300679</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
       <c r="E11" t="n">
         <v>0.2</v>
       </c>
@@ -1595,7 +1559,6 @@
           <t>sz300442</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
       <c r="E12" t="n">
         <v>0.25</v>
       </c>
@@ -1616,7 +1579,6 @@
           <t>sh600588</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
       <c r="E13" t="n">
         <v>0.25</v>
       </c>
@@ -1637,7 +1599,6 @@
           <t>sh603039</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
       <c r="E14" t="n">
         <v>0.25</v>
       </c>
@@ -1658,7 +1619,6 @@
           <t>sz300383</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
       <c r="E15" t="n">
         <v>0.25</v>
       </c>
@@ -1679,7 +1639,6 @@
           <t>sh600536</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
       <c r="E16" t="n">
         <v>0.25</v>
       </c>
@@ -1700,7 +1659,6 @@
           <t>sz002230</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
       <c r="E17" t="n">
         <v>0.25</v>
       </c>
@@ -1721,7 +1679,6 @@
           <t>sz300454</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
       <c r="E18" t="n">
         <v>0.25</v>
       </c>
@@ -1742,7 +1699,6 @@
           <t>sh600588</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
       <c r="E19" t="n">
         <v>0.25</v>
       </c>
@@ -1763,7 +1719,6 @@
           <t>sh600637</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
       <c r="E20" t="n">
         <v>0.25</v>
       </c>
@@ -1784,7 +1739,6 @@
           <t>sz300418</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
       <c r="E21" t="n">
         <v>0.25</v>
       </c>
@@ -1805,7 +1759,6 @@
           <t>sh603888</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
       <c r="E22" t="n">
         <v>0.25</v>
       </c>
@@ -1826,7 +1779,6 @@
           <t>sz002624</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr"/>
       <c r="E23" t="n">
         <v>0.25</v>
       </c>
@@ -1847,7 +1799,6 @@
           <t>sh603019</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr"/>
       <c r="E24" t="n">
         <v>0.3333</v>
       </c>
@@ -1868,7 +1819,6 @@
           <t>sz300659</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr"/>
       <c r="E25" t="n">
         <v>0.3333</v>
       </c>
@@ -1889,7 +1839,6 @@
           <t>sz300168</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr"/>
       <c r="E26" t="n">
         <v>0.3333</v>
       </c>
@@ -1910,7 +1859,6 @@
           <t>sz002475</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr"/>
       <c r="E27" t="n">
         <v>0.25</v>
       </c>
@@ -1931,7 +1879,6 @@
           <t>sh603501</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr"/>
       <c r="E28" t="n">
         <v>0.25</v>
       </c>
@@ -1952,7 +1899,6 @@
           <t>sz300136</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr"/>
       <c r="E29" t="n">
         <v>0.25</v>
       </c>
@@ -1973,7 +1919,6 @@
           <t>sz002916</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr"/>
       <c r="E30" t="n">
         <v>0.25</v>
       </c>
@@ -1994,7 +1939,6 @@
           <t>sh601012</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr"/>
       <c r="E31" t="n">
         <v>0.25</v>
       </c>
@@ -2015,7 +1959,6 @@
           <t>sz300750</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr"/>
       <c r="E32" t="n">
         <v>0.25</v>
       </c>
@@ -2036,7 +1979,6 @@
           <t>sz002129</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr"/>
       <c r="E33" t="n">
         <v>0.25</v>
       </c>
@@ -2057,7 +1999,6 @@
           <t>sh600438</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr"/>
       <c r="E34" t="n">
         <v>0.25</v>
       </c>
@@ -2078,7 +2019,6 @@
           <t>sz002594</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr"/>
       <c r="E35" t="n">
         <v>0.25</v>
       </c>
@@ -2099,7 +2039,6 @@
           <t>sh600104</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr"/>
       <c r="E36" t="n">
         <v>0.25</v>
       </c>
@@ -2120,7 +2059,6 @@
           <t>sh601633</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr"/>
       <c r="E37" t="n">
         <v>0.25</v>
       </c>
@@ -2141,7 +2079,6 @@
           <t>sz000625</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr"/>
       <c r="E38" t="n">
         <v>0.25</v>
       </c>
@@ -2162,7 +2099,6 @@
           <t>sz300750</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr"/>
       <c r="E39" t="n">
         <v>0.25</v>
       </c>
@@ -2183,7 +2119,6 @@
           <t>sz002074</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr"/>
       <c r="E40" t="n">
         <v>0.25</v>
       </c>
@@ -2204,7 +2139,6 @@
           <t>sh600884</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr"/>
       <c r="E41" t="n">
         <v>0.25</v>
       </c>
@@ -2225,7 +2159,6 @@
           <t>sz002709</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr"/>
       <c r="E42" t="n">
         <v>0.25</v>
       </c>
@@ -2246,7 +2179,6 @@
           <t>sh601012</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr"/>
       <c r="E43" t="n">
         <v>0.25</v>
       </c>
@@ -2267,7 +2199,6 @@
           <t>sh600438</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr"/>
       <c r="E44" t="n">
         <v>0.25</v>
       </c>
@@ -2288,7 +2219,6 @@
           <t>sz300274</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr"/>
       <c r="E45" t="n">
         <v>0.25</v>
       </c>
@@ -2309,7 +2239,6 @@
           <t>sh688599</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr"/>
       <c r="E46" t="n">
         <v>0.25</v>
       </c>
@@ -2330,7 +2259,6 @@
           <t>sh601398</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr"/>
       <c r="E47" t="n">
         <v>0.25</v>
       </c>
@@ -2351,7 +2279,6 @@
           <t>sh601939</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr"/>
       <c r="E48" t="n">
         <v>0.25</v>
       </c>
@@ -2372,7 +2299,6 @@
           <t>sh600036</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr"/>
       <c r="E49" t="n">
         <v>0.25</v>
       </c>
@@ -2393,7 +2319,6 @@
           <t>sh601166</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr"/>
       <c r="E50" t="n">
         <v>0.25</v>
       </c>
@@ -2414,7 +2339,6 @@
           <t>sh601318</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr"/>
       <c r="E51" t="n">
         <v>0.25</v>
       </c>
@@ -2435,7 +2359,6 @@
           <t>sh601628</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr"/>
       <c r="E52" t="n">
         <v>0.25</v>
       </c>
@@ -2456,7 +2379,6 @@
           <t>sh601601</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr"/>
       <c r="E53" t="n">
         <v>0.25</v>
       </c>
@@ -2477,7 +2399,6 @@
           <t>sh601336</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr"/>
       <c r="E54" t="n">
         <v>0.25</v>
       </c>
@@ -2498,7 +2419,6 @@
           <t>sh600030</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr"/>
       <c r="E55" t="n">
         <v>0.25</v>
       </c>
@@ -2519,7 +2439,6 @@
           <t>sh601211</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr"/>
       <c r="E56" t="n">
         <v>0.25</v>
       </c>
@@ -2540,7 +2459,6 @@
           <t>sz002736</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr"/>
       <c r="E57" t="n">
         <v>0.25</v>
       </c>
@@ -2561,7 +2479,6 @@
           <t>sh600837</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr"/>
       <c r="E58" t="n">
         <v>0.25</v>
       </c>
@@ -2582,7 +2499,6 @@
           <t>sh688981</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr"/>
       <c r="E59" t="n">
         <v>0.25</v>
       </c>
@@ -2603,7 +2519,6 @@
           <t>sz300760</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr"/>
       <c r="E60" t="n">
         <v>0.25</v>
       </c>
@@ -2624,7 +2539,6 @@
           <t>sz300003</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr"/>
       <c r="E61" t="n">
         <v>0.25</v>
       </c>
@@ -2645,7 +2559,6 @@
           <t>sh603259</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr"/>
       <c r="E62" t="n">
         <v>0.25</v>
       </c>
@@ -2666,7 +2579,6 @@
           <t>sh600276</t>
         </is>
       </c>
-      <c r="D63" t="inlineStr"/>
       <c r="E63" t="n">
         <v>0.25</v>
       </c>
@@ -2687,7 +2599,6 @@
           <t>sz300015</t>
         </is>
       </c>
-      <c r="D64" t="inlineStr"/>
       <c r="E64" t="n">
         <v>0.25</v>
       </c>
@@ -2708,7 +2619,6 @@
           <t>sh600196</t>
         </is>
       </c>
-      <c r="D65" t="inlineStr"/>
       <c r="E65" t="n">
         <v>0.25</v>
       </c>
@@ -2729,7 +2639,6 @@
           <t>sz000538</t>
         </is>
       </c>
-      <c r="D66" t="inlineStr"/>
       <c r="E66" t="n">
         <v>0.25</v>
       </c>
@@ -2750,7 +2659,6 @@
           <t>sz300760</t>
         </is>
       </c>
-      <c r="D67" t="inlineStr"/>
       <c r="E67" t="n">
         <v>0.25</v>
       </c>
@@ -2771,7 +2679,6 @@
           <t>sz300003</t>
         </is>
       </c>
-      <c r="D68" t="inlineStr"/>
       <c r="E68" t="n">
         <v>0.25</v>
       </c>
@@ -2792,7 +2699,6 @@
           <t>sh688016</t>
         </is>
       </c>
-      <c r="D69" t="inlineStr"/>
       <c r="E69" t="n">
         <v>0.25</v>
       </c>
@@ -2813,7 +2719,6 @@
           <t>sz002223</t>
         </is>
       </c>
-      <c r="D70" t="inlineStr"/>
       <c r="E70" t="n">
         <v>0.25</v>
       </c>
@@ -2834,7 +2739,6 @@
           <t>sh600519</t>
         </is>
       </c>
-      <c r="D71" t="inlineStr"/>
       <c r="E71" t="n">
         <v>0.25</v>
       </c>
@@ -2855,7 +2759,6 @@
           <t>sh000858</t>
         </is>
       </c>
-      <c r="D72" t="inlineStr"/>
       <c r="E72" t="n">
         <v>0.25</v>
       </c>
@@ -2876,7 +2779,6 @@
           <t>sz002304</t>
         </is>
       </c>
-      <c r="D73" t="inlineStr"/>
       <c r="E73" t="n">
         <v>0.25</v>
       </c>
@@ -2897,7 +2799,6 @@
           <t>sh600887</t>
         </is>
       </c>
-      <c r="D74" t="inlineStr"/>
       <c r="E74" t="n">
         <v>0.25</v>
       </c>
@@ -2918,7 +2819,6 @@
           <t>sh600519</t>
         </is>
       </c>
-      <c r="D75" t="inlineStr"/>
       <c r="E75" t="n">
         <v>0.25</v>
       </c>
@@ -2939,7 +2839,6 @@
           <t>sh600887</t>
         </is>
       </c>
-      <c r="D76" t="inlineStr"/>
       <c r="E76" t="n">
         <v>0.25</v>
       </c>
@@ -2960,7 +2859,6 @@
           <t>sz000858</t>
         </is>
       </c>
-      <c r="D77" t="inlineStr"/>
       <c r="E77" t="n">
         <v>0.25</v>
       </c>
@@ -2981,7 +2879,6 @@
           <t>sh603288</t>
         </is>
       </c>
-      <c r="D78" t="inlineStr"/>
       <c r="E78" t="n">
         <v>0.25</v>
       </c>
@@ -3002,7 +2899,6 @@
           <t>sz002024</t>
         </is>
       </c>
-      <c r="D79" t="inlineStr"/>
       <c r="E79" t="n">
         <v>0.25</v>
       </c>
@@ -3023,7 +2919,6 @@
           <t>sh600827</t>
         </is>
       </c>
-      <c r="D80" t="inlineStr"/>
       <c r="E80" t="n">
         <v>0.25</v>
       </c>
@@ -3044,7 +2939,6 @@
           <t>sh601933</t>
         </is>
       </c>
-      <c r="D81" t="inlineStr"/>
       <c r="E81" t="n">
         <v>0.25</v>
       </c>
@@ -3065,7 +2959,6 @@
           <t>sz300413</t>
         </is>
       </c>
-      <c r="D82" t="inlineStr"/>
       <c r="E82" t="n">
         <v>0.25</v>
       </c>
@@ -3086,7 +2979,6 @@
           <t>sh600760</t>
         </is>
       </c>
-      <c r="D83" t="inlineStr"/>
       <c r="E83" t="n">
         <v>0.25</v>
       </c>
@@ -3107,7 +2999,6 @@
           <t>sh600893</t>
         </is>
       </c>
-      <c r="D84" t="inlineStr"/>
       <c r="E84" t="n">
         <v>0.25</v>
       </c>
@@ -3128,7 +3019,6 @@
           <t>sz000768</t>
         </is>
       </c>
-      <c r="D85" t="inlineStr"/>
       <c r="E85" t="n">
         <v>0.25</v>
       </c>
@@ -3149,7 +3039,6 @@
           <t>sh600862</t>
         </is>
       </c>
-      <c r="D86" t="inlineStr"/>
       <c r="E86" t="n">
         <v>0.25</v>
       </c>
@@ -3170,7 +3059,6 @@
           <t>sh600760</t>
         </is>
       </c>
-      <c r="D87" t="inlineStr"/>
       <c r="E87" t="n">
         <v>0.25</v>
       </c>
@@ -3191,7 +3079,6 @@
           <t>sh600893</t>
         </is>
       </c>
-      <c r="D88" t="inlineStr"/>
       <c r="E88" t="n">
         <v>0.25</v>
       </c>
@@ -3212,7 +3099,6 @@
           <t>sz000768</t>
         </is>
       </c>
-      <c r="D89" t="inlineStr"/>
       <c r="E89" t="n">
         <v>0.25</v>
       </c>
@@ -3233,7 +3119,6 @@
           <t>sh600185</t>
         </is>
       </c>
-      <c r="D90" t="inlineStr"/>
       <c r="E90" t="n">
         <v>0.25</v>
       </c>
@@ -3254,7 +3139,6 @@
           <t>sz300124</t>
         </is>
       </c>
-      <c r="D91" t="inlineStr"/>
       <c r="E91" t="n">
         <v>0.25</v>
       </c>
@@ -3275,7 +3159,6 @@
           <t>sh601100</t>
         </is>
       </c>
-      <c r="D92" t="inlineStr"/>
       <c r="E92" t="n">
         <v>0.25</v>
       </c>
@@ -3296,7 +3179,6 @@
           <t>sz300024</t>
         </is>
       </c>
-      <c r="D93" t="inlineStr"/>
       <c r="E93" t="n">
         <v>0.25</v>
       </c>
@@ -3317,7 +3199,6 @@
           <t>sz002747</t>
         </is>
       </c>
-      <c r="D94" t="inlineStr"/>
       <c r="E94" t="n">
         <v>0.25</v>
       </c>
@@ -3338,7 +3219,6 @@
           <t>sh600028</t>
         </is>
       </c>
-      <c r="D95" t="inlineStr"/>
       <c r="E95" t="n">
         <v>0.25</v>
       </c>
@@ -3359,7 +3239,6 @@
           <t>sh601857</t>
         </is>
       </c>
-      <c r="D96" t="inlineStr"/>
       <c r="E96" t="n">
         <v>0.25</v>
       </c>
@@ -3380,7 +3259,6 @@
           <t>sh600256</t>
         </is>
       </c>
-      <c r="D97" t="inlineStr"/>
       <c r="E97" t="n">
         <v>0.25</v>
       </c>
@@ -3401,7 +3279,6 @@
           <t>sh600688</t>
         </is>
       </c>
-      <c r="D98" t="inlineStr"/>
       <c r="E98" t="n">
         <v>0.25</v>
       </c>
@@ -3422,7 +3299,6 @@
           <t>sh601600</t>
         </is>
       </c>
-      <c r="D99" t="inlineStr"/>
       <c r="E99" t="n">
         <v>0.25</v>
       </c>
@@ -3443,7 +3319,6 @@
           <t>sh600362</t>
         </is>
       </c>
-      <c r="D100" t="inlineStr"/>
       <c r="E100" t="n">
         <v>0.25</v>
       </c>
@@ -3464,7 +3339,6 @@
           <t>sz000630</t>
         </is>
       </c>
-      <c r="D101" t="inlineStr"/>
       <c r="E101" t="n">
         <v>0.25</v>
       </c>
@@ -3485,7 +3359,6 @@
           <t>sh600547</t>
         </is>
       </c>
-      <c r="D102" t="inlineStr"/>
       <c r="E102" t="n">
         <v>0.25</v>
       </c>
@@ -3506,7 +3379,6 @@
           <t>sh600019</t>
         </is>
       </c>
-      <c r="D103" t="inlineStr"/>
       <c r="E103" t="n">
         <v>0.25</v>
       </c>
@@ -3527,7 +3399,6 @@
           <t>sh600010</t>
         </is>
       </c>
-      <c r="D104" t="inlineStr"/>
       <c r="E104" t="n">
         <v>0.25</v>
       </c>
@@ -3548,7 +3419,6 @@
           <t>sz000708</t>
         </is>
       </c>
-      <c r="D105" t="inlineStr"/>
       <c r="E105" t="n">
         <v>0.25</v>
       </c>
@@ -3569,7 +3439,6 @@
           <t>sh600808</t>
         </is>
       </c>
-      <c r="D106" t="inlineStr"/>
       <c r="E106" t="n">
         <v>0.25</v>
       </c>
@@ -3590,7 +3459,6 @@
           <t>sh601088</t>
         </is>
       </c>
-      <c r="D107" t="inlineStr"/>
       <c r="E107" t="n">
         <v>0.25</v>
       </c>
@@ -3611,7 +3479,6 @@
           <t>sh600188</t>
         </is>
       </c>
-      <c r="D108" t="inlineStr"/>
       <c r="E108" t="n">
         <v>0.25</v>
       </c>
@@ -3632,7 +3499,6 @@
           <t>sh600546</t>
         </is>
       </c>
-      <c r="D109" t="inlineStr"/>
       <c r="E109" t="n">
         <v>0.25</v>
       </c>
@@ -3653,7 +3519,6 @@
           <t>sz000983</t>
         </is>
       </c>
-      <c r="D110" t="inlineStr"/>
       <c r="E110" t="n">
         <v>0.25</v>
       </c>
@@ -3674,7 +3539,6 @@
           <t>sh601668</t>
         </is>
       </c>
-      <c r="D111" t="inlineStr"/>
       <c r="E111" t="n">
         <v>0.25</v>
       </c>
@@ -3695,7 +3559,6 @@
           <t>sh601186</t>
         </is>
       </c>
-      <c r="D112" t="inlineStr"/>
       <c r="E112" t="n">
         <v>0.25</v>
       </c>
@@ -3716,7 +3579,6 @@
           <t>sh601390</t>
         </is>
       </c>
-      <c r="D113" t="inlineStr"/>
       <c r="E113" t="n">
         <v>0.25</v>
       </c>
@@ -3737,7 +3599,6 @@
           <t>sh600585</t>
         </is>
       </c>
-      <c r="D114" t="inlineStr"/>
       <c r="E114" t="n">
         <v>0.25</v>
       </c>
@@ -3758,7 +3619,6 @@
           <t>sh600048</t>
         </is>
       </c>
-      <c r="D115" t="inlineStr"/>
       <c r="E115" t="n">
         <v>0.25</v>
       </c>
@@ -3779,7 +3639,6 @@
           <t>sz000002</t>
         </is>
       </c>
-      <c r="D116" t="inlineStr"/>
       <c r="E116" t="n">
         <v>0.25</v>
       </c>
@@ -3800,7 +3659,6 @@
           <t>sh600383</t>
         </is>
       </c>
-      <c r="D117" t="inlineStr"/>
       <c r="E117" t="n">
         <v>0.25</v>
       </c>
@@ -3821,7 +3679,6 @@
           <t>sh600340</t>
         </is>
       </c>
-      <c r="D118" t="inlineStr"/>
       <c r="E118" t="n">
         <v>0.25</v>
       </c>
@@ -3842,7 +3699,6 @@
           <t>sh600233</t>
         </is>
       </c>
-      <c r="D119" t="inlineStr"/>
       <c r="E119" t="n">
         <v>0.25</v>
       </c>
@@ -3863,7 +3719,6 @@
           <t>sz002120</t>
         </is>
       </c>
-      <c r="D120" t="inlineStr"/>
       <c r="E120" t="n">
         <v>0.25</v>
       </c>
@@ -3884,7 +3739,6 @@
           <t>sh600029</t>
         </is>
       </c>
-      <c r="D121" t="inlineStr"/>
       <c r="E121" t="n">
         <v>0.25</v>
       </c>
@@ -3905,7 +3759,6 @@
           <t>sh601111</t>
         </is>
       </c>
-      <c r="D122" t="inlineStr"/>
       <c r="E122" t="n">
         <v>0.25</v>
       </c>
@@ -3926,7 +3779,6 @@
           <t>sz002714</t>
         </is>
       </c>
-      <c r="D123" t="inlineStr"/>
       <c r="E123" t="n">
         <v>0.5</v>
       </c>
@@ -3947,7 +3799,6 @@
           <t>sz002157</t>
         </is>
       </c>
-      <c r="D124" t="inlineStr"/>
       <c r="E124" t="n">
         <v>0.5</v>
       </c>
@@ -3966,10 +3817,10 @@
   <dimension ref="A1:D40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
-    <col width="35" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="72" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3988,13 +3839,13 @@
           <t>Default</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="36" customHeight="1">
       <c r="A2" t="inlineStr">
         <is>
           <t>us_min_gain_5d</t>
@@ -4010,13 +3861,13 @@
           <t>3.0</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>FILTER_CONFIG parameter</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>板块联动筛选阈值：美股对应板块近5个交易日涨幅至少达到该百分比，才认为美股端有短线强势信号。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="36" customHeight="1">
       <c r="A3" t="inlineStr">
         <is>
           <t>us_min_gain_20d</t>
@@ -4032,13 +3883,13 @@
           <t>5.0</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>FILTER_CONFIG parameter</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>板块联动筛选阈值：美股对应板块近20个交易日涨幅至少达到该百分比，用于确认中期强势趋势。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="36" customHeight="1">
       <c r="A4" t="inlineStr">
         <is>
           <t>cn_max_gain_5d</t>
@@ -4054,13 +3905,13 @@
           <t>1.0</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>FILTER_CONFIG parameter</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>板块联动筛选阈值：A股对应板块近5个交易日涨幅不高于该百分比，用于寻找短线滞涨板块。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="36" customHeight="1">
       <c r="A5" t="inlineStr">
         <is>
           <t>cn_max_gain_20d</t>
@@ -4076,13 +3927,13 @@
           <t>2.0</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>FILTER_CONFIG parameter</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>板块联动筛选阈值：A股对应板块近20个交易日涨幅不高于该百分比，用于寻找中期滞涨板块。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="36" customHeight="1">
       <c r="A6" t="inlineStr">
         <is>
           <t>min_gap_5d</t>
@@ -4098,13 +3949,13 @@
           <t>3.0</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>FILTER_CONFIG parameter</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>中美板块背离阈值：美股5日涨幅减A股5日涨幅的最小差值，差值越大代表A股补涨空间越明显。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="36" customHeight="1">
       <c r="A7" t="inlineStr">
         <is>
           <t>min_gap_20d</t>
@@ -4120,13 +3971,13 @@
           <t>5.0</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>FILTER_CONFIG parameter</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>中美板块背离阈值：美股20日涨幅减A股20日涨幅的最小差值，用于衡量中期补涨机会。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="36" customHeight="1">
       <c r="A8" t="inlineStr">
         <is>
           <t>div_us20</t>
@@ -4142,13 +3993,13 @@
           <t>5.0</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>背离筛选：美股20日最低涨幅(%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>背离筛选参数：美股板块20日涨幅需不低于该百分比，作为海外端强势确认条件。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="36" customHeight="1">
       <c r="A9" t="inlineStr">
         <is>
           <t>div_cn20</t>
@@ -4164,13 +4015,13 @@
           <t>2.0</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>背离筛选：A股20日最高涨幅(%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>背离筛选参数：A股板块20日涨幅需不高于该百分比，作为国内端尚未充分跟涨的条件。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="36" customHeight="1">
       <c r="A10" t="inlineStr">
         <is>
           <t>div_us5</t>
@@ -4186,13 +4037,13 @@
           <t>3.0</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>背离筛选：美股5日最低涨幅(%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>背离筛选参数：美股板块5日涨幅需不低于该百分比，用于捕捉近期催化和短线强势。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="36" customHeight="1">
       <c r="A11" t="inlineStr">
         <is>
           <t>request_retry_max</t>
@@ -4208,13 +4059,13 @@
           <t>3</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>FILTER_CONFIG parameter</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>数据请求容错参数：单个接口请求失败后的最大重试次数。</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="36" customHeight="1">
       <c r="A12" t="inlineStr">
         <is>
           <t>request_retry_delay</t>
@@ -4230,13 +4081,13 @@
           <t>0.8</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>FILTER_CONFIG parameter</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>数据请求容错参数：失败重试前的等待秒数，避免连续请求过快。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="36" customHeight="1">
       <c r="A13" t="inlineStr">
         <is>
           <t>request_delay</t>
@@ -4252,13 +4103,13 @@
           <t>0.25</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>FILTER_CONFIG parameter</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>数据请求节流参数：正常请求之间的等待秒数，用于降低触发限流的概率。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="36" customHeight="1">
       <c r="A14" t="inlineStr">
         <is>
           <t>sector_cache_ttl_hours</t>
@@ -4274,13 +4125,13 @@
           <t>1</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>FILTER_CONFIG parameter</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>板块数据缓存有效期，单位为小时；缓存未过期时优先复用本地结果。</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="36" customHeight="1">
       <c r="A15" t="inlineStr">
         <is>
           <t>stock_score_threshold</t>
@@ -4296,13 +4147,13 @@
           <t>60</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>FILTER_CONFIG parameter</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>个股入选分数线：综合技术面、量能、支撑等指标后的最低通过分。</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="36" customHeight="1">
       <c r="A16" t="inlineStr">
         <is>
           <t>max_stocks_per_sector</t>
@@ -4318,13 +4169,13 @@
           <t>10</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>FILTER_CONFIG parameter</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>每个板块最多保留的候选股票数量，用于控制输出列表长度。</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="36" customHeight="1">
       <c r="A17" t="inlineStr">
         <is>
           <t>macd_fast</t>
@@ -4340,13 +4191,13 @@
           <t>12</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>FILTER_CONFIG parameter</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>日线MACD快线EMA周期，通常为12；用于计算DIF中的短周期均线。</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="36" customHeight="1">
       <c r="A18" t="inlineStr">
         <is>
           <t>macd_slow</t>
@@ -4362,13 +4213,13 @@
           <t>26</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>FILTER_CONFIG parameter</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>日线MACD慢线EMA周期，通常为26；用于计算DIF中的长周期均线。</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="36" customHeight="1">
       <c r="A19" t="inlineStr">
         <is>
           <t>macd_signal</t>
@@ -4384,13 +4235,13 @@
           <t>9</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>FILTER_CONFIG parameter</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>日线MACD信号线DEA周期，通常为9；用于判断MACD金叉、死叉和柱体变化。</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="36" customHeight="1">
       <c r="A20" t="inlineStr">
         <is>
           <t>support_resistance_lookback</t>
@@ -4406,13 +4257,13 @@
           <t>60</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>FILTER_CONFIG parameter</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>支撑/压力识别回看窗口，单位为交易日；用于寻找近期高低点、平台和关键价位。</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="36" customHeight="1">
       <c r="A21" t="inlineStr">
         <is>
           <t>weekly_macd_fast</t>
@@ -4428,13 +4279,13 @@
           <t>12</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>FILTER_CONFIG parameter</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>周线MACD快线EMA周期，用于从更高周期确认趋势强弱。</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="36" customHeight="1">
       <c r="A22" t="inlineStr">
         <is>
           <t>weekly_macd_slow</t>
@@ -4450,13 +4301,13 @@
           <t>26</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>FILTER_CONFIG parameter</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>周线MACD慢线EMA周期，用于周线DIF计算并过滤短期噪声。</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="36" customHeight="1">
       <c r="A23" t="inlineStr">
         <is>
           <t>weekly_macd_signal</t>
@@ -4472,13 +4323,13 @@
           <t>9</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>FILTER_CONFIG parameter</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>周线MACD信号线DEA周期，用于判断周线级别的趋势拐点。</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="36" customHeight="1">
       <c r="A24" t="inlineStr">
         <is>
           <t>weekly_green_shorten_weeks</t>
@@ -4494,13 +4345,13 @@
           <t>2</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>FILTER_CONFIG parameter</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>周线MACD绿柱连续缩短的最少周数；满足时代表空头动能减弱。</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="36" customHeight="1">
       <c r="A25" t="inlineStr">
         <is>
           <t>weekly_red_lengthen_weeks</t>
@@ -4516,13 +4367,13 @@
           <t>2</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>FILTER_CONFIG parameter</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>周线MACD红柱连续放大的最少周数；满足时代表多头动能增强。</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="36" customHeight="1">
       <c r="A26" t="inlineStr">
         <is>
           <t>weekly_min_history_weeks</t>
@@ -4538,13 +4389,13 @@
           <t>52</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>FILTER_CONFIG parameter</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>周线技术指标所需的最少历史周数；历史不足时周线判断可信度降低。</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="36" customHeight="1">
       <c r="A27" t="inlineStr">
         <is>
           <t>fib_levels</t>
@@ -4560,13 +4411,13 @@
           <t>[0.236, 0.382, 0.5, 0.618, 0.786]</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>FILTER_CONFIG parameter</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>斐波那契回撤/反弹比例集合，用于计算潜在支撑位、压力位和回撤目标。</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="36" customHeight="1">
       <c r="A28" t="inlineStr">
         <is>
           <t>pivot_lookback_weeks</t>
@@ -4582,13 +4433,13 @@
           <t>20</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>FILTER_CONFIG parameter</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>周线枢轴点识别回看窗口，单位为周；用于寻找阶段性高点、低点和结构位置。</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="36" customHeight="1">
       <c r="A29" t="inlineStr">
         <is>
           <t>ma_support_periods</t>
@@ -4604,13 +4455,13 @@
           <t>[20, 60]</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>FILTER_CONFIG parameter</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>均线支撑周期列表，例如20日、60日；价格靠近这些均线时可视为潜在支撑测试。</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="36" customHeight="1">
       <c r="A30" t="inlineStr">
         <is>
           <t>volume_confirmation_days</t>
@@ -4626,13 +4477,13 @@
           <t>5</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>FILTER_CONFIG parameter</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>量能确认窗口，单位为交易日；用于比较近期成交量是否配合价格信号。</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="36" customHeight="1">
       <c r="A31" t="inlineStr">
         <is>
           <t>support_confluence_tolerance</t>
@@ -4648,13 +4499,13 @@
           <t>0.02</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>FILTER_CONFIG parameter</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>支撑共振容差比例；多个支撑位距离当前价在该比例以内时视为同一区域。</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="36" customHeight="1">
       <c r="A32" t="inlineStr">
         <is>
           <t>confidence_weight_yfinance</t>
@@ -4670,13 +4521,13 @@
           <t>0.4</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>FILTER_CONFIG parameter</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>跨数据源置信度权重：yfinance数据在综合置信度中的占比。</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="36" customHeight="1">
       <c r="A33" t="inlineStr">
         <is>
           <t>confidence_weight_sina</t>
@@ -4692,13 +4543,13 @@
           <t>0.3</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>FILTER_CONFIG parameter</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>跨数据源置信度权重：新浪数据在综合置信度中的占比。</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="36" customHeight="1">
       <c r="A34" t="inlineStr">
         <is>
           <t>confidence_weight_eastmoney</t>
@@ -4714,13 +4565,13 @@
           <t>0.3</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>FILTER_CONFIG parameter</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>跨数据源置信度权重：东方财富数据在综合置信度中的占比。</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="36" customHeight="1">
       <c r="A35" t="inlineStr">
         <is>
           <t>min_confidence_score</t>
@@ -4736,13 +4587,13 @@
           <t>0.6</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>FILTER_CONFIG parameter</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>数据交叉验证最低置信度；低于该分数的行情或指标结果不建议进入最终筛选。</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="36" customHeight="1">
       <c r="A36" t="inlineStr">
         <is>
           <t>cross_validate_tolerance</t>
@@ -4758,13 +4609,13 @@
           <t>0.05</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>FILTER_CONFIG parameter</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>跨数据源价格/涨跌幅允许误差比例；超过该容差时认为数据源之间存在冲突。</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="36" customHeight="1">
       <c r="A37" t="inlineStr">
         <is>
           <t>exclude_st_stocks</t>
@@ -4780,13 +4631,13 @@
           <t>True</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>FILTER_CONFIG parameter</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>风险过滤开关：为True时排除ST、*ST等风险警示股票。</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="36" customHeight="1">
       <c r="A38" t="inlineStr">
         <is>
           <t>exclude_new_stocks_days</t>
@@ -4802,13 +4653,13 @@
           <t>60</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>FILTER_CONFIG parameter</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>新股过滤窗口，单位为自然日或交易日口径依实现而定；上市时间短于该值的股票会被排除。</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="36" customHeight="1">
       <c r="A39" t="inlineStr">
         <is>
           <t>max_decline_ratio</t>
@@ -4824,13 +4675,13 @@
           <t>-0.15</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>FILTER_CONFIG parameter</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>风险过滤阈值：允许的最大阶段跌幅比例；跌幅超过该负值阈值时剔除弱势或破位个股。</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="36" customHeight="1">
       <c r="A40" t="inlineStr">
         <is>
           <t>min_volume_ratio</t>
@@ -4846,9 +4697,9 @@
           <t>0.3</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>FILTER_CONFIG parameter</t>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>流动性过滤阈值：成交量相对基准量能的最低比例，低于该值说明交易活跃度不足。</t>
         </is>
       </c>
     </row>

</xml_diff>